<commit_message>
update reg files for mental health and wellbeing
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dasha\ESSEX\_SimPaths\_SimPaths_UK\input_processing\regression_estimates\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\simpaths_dev\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD2E4EB-0516-4B27-A05C-B535DEC893B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496F0204-32B2-4494-AB59-B58547A7709A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -64,43 +64,13 @@
     <t>HM1_L</t>
   </si>
   <si>
-    <t>HM2_Females_L</t>
-  </si>
-  <si>
-    <t>HM2_Males_L</t>
-  </si>
-  <si>
-    <t>HM2_Females_C</t>
-  </si>
-  <si>
-    <t>HM2_Males_C</t>
-  </si>
-  <si>
     <t>DHE_MCS1</t>
   </si>
   <si>
-    <t>DHE_MCS2_Females</t>
-  </si>
-  <si>
-    <t>DHE_MCS2_Males</t>
-  </si>
-  <si>
     <t>DHE_PCS1</t>
   </si>
   <si>
-    <t>DHE_PCS2_Females</t>
-  </si>
-  <si>
-    <t>DHE_PCS2_Males</t>
-  </si>
-  <si>
     <t>DLS1</t>
-  </si>
-  <si>
-    <t>DLS2_Females</t>
-  </si>
-  <si>
-    <t>DLS2_Males</t>
   </si>
 </sst>
 </file>
@@ -469,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.140625" customWidth="1"/>
@@ -576,7 +546,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>4.4608727317206842</v>
+        <v>4.1855465085565644</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -584,7 +554,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>4.2488100047405588</v>
+        <v>7.4908409588260065</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -592,7 +562,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>3.7376343170238648</v>
+        <v>7.4908409588260065</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -600,87 +570,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>2.5968664130199306</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17">
-        <v>2.1885543164797094</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18">
-        <v>7.966919324090096</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19">
-        <v>7.1657841258237269</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20">
-        <v>6.4859586641425091</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21">
-        <v>7.0661394726712041</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22">
-        <v>6.0523880929117633</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23">
-        <v>5.4222029042219946</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24">
-        <v>1.902513219539105</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25">
-        <v>1.7134881680118068</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>26</v>
-      </c>
-      <c r="B26">
-        <v>1.6261256004830791</v>
+        <v>1.8161778493855598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>